<commit_message>
Methodik-Berichte #96/#98 (risiko-auto, abnahmereif) + PDF-Export-Pipeline + Doku-/WIP-Stände
- docs/methodik/96_aeroallergene.md + 98_uv_schaedigungen.md (§4-Format, je 3
  Review-Runden bis Null-Runde; Ledger reviews/BEFUNDE_96/98.md; Lese-PDFs)
- Herleitungsskripte + Ergebnisdaten: dwd_pollensaison.py (Saison-Spreizung aus
  DWD-Phänologie), dwd_ssd_trend.py (SSD-Normalperioden + k_UV-Kette),
  kid2025_ablesewerte.csv; zentrales Evidenz-Register erweitert (#96/#98-Zeilen)
- PDF-Export umgestellt: pandoc→KaTeX-HTML→Playwright-Chromium (M0-Optik;
  scripts/export_methodik_pdf.sh, methodik_report.css, html_to_pdf.py)
- Aufgabe v2, Commands (.claude/), M0-Render/Archiv, Roadmap-Seiten und weitere
  offene Arbeitsstände (Backend/Frontend) mit eingecheckt

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012v8KP7fKiu2jYq4n1StAqw
</commit_message>
<xml_diff>
--- a/docs/Schadensbaum/KWRA-Monetarisierung.xlsx
+++ b/docs/Schadensbaum/KWRA-Monetarisierung.xlsx
@@ -803,37 +803,37 @@
           <t>Handlungserfordernis</t>
         </is>
       </c>
-      <c r="H5" s="31" t="inlineStr">
+      <c r="H5" s="32" t="inlineStr">
         <is>
           <t>Rolle in der Monetarisierung</t>
         </is>
       </c>
-      <c r="I5" s="31" t="inlineStr">
+      <c r="I5" s="32" t="inlineStr">
         <is>
           <t>Schadenskonto</t>
         </is>
       </c>
-      <c r="J5" s="31" t="inlineStr">
+      <c r="J5" s="32" t="inlineStr">
         <is>
           <t>Bewertungsansatz / Kostensatz</t>
         </is>
       </c>
-      <c r="K5" s="31" t="inlineStr">
+      <c r="K5" s="32" t="inlineStr">
         <is>
           <t>Wird hier bepreist (enthalten)</t>
         </is>
       </c>
-      <c r="L5" s="31" t="inlineStr">
+      <c r="L5" s="32" t="inlineStr">
         <is>
           <t>Nicht enthalten (gebucht in …)</t>
         </is>
       </c>
-      <c r="M5" s="31" t="inlineStr">
+      <c r="M5" s="32" t="inlineStr">
         <is>
           <t>Wirkt über / bucht in (IDs, Konten)</t>
         </is>
       </c>
-      <c r="N5" s="31" t="inlineStr">
+      <c r="N5" s="32" t="inlineStr">
         <is>
           <t>Regeln</t>
         </is>
@@ -7763,7 +7763,7 @@
       </c>
       <c r="J100" s="35" t="inlineStr">
         <is>
-          <t>Mortalität: hitzebedingte Übersterblichkeit × VSL (Nutzer-Setzung 3,5 Mio. €/Fall; Quelle für offizielle Sätze: UBA-Methodenkonvention). Morbidität: Fallzahlen × Behandlungskostensätze. K1 ist nach Ursachen partitioniert (R9): jeder Todesfall zählt genau einmal.</t>
+          <t>Mortalität: hitzebedingte Übersterblichkeit als YLL × VOLY (MK 4.0; VSL nur Sensitivität — Fortschreibung P52). Morbidität: Fallzahlen × Behandlungskostensätze. K1 ist nach Ursachen partitioniert (R9): jeder Todesfall zählt genau einmal.</t>
         </is>
       </c>
       <c r="K100" s="35" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="J103" s="41" t="inlineStr">
         <is>
-          <t>Zusätzliche Erkrankungsfälle × Behandlungskosten + Mortalitätsanteil × VSL.</t>
+          <t>Zusätzliche Erkrankungsfälle × Behandlungskosten + Mortalitätsanteil als YLL × VOLY (MK 4.0; VSL nur Sensitivität — Fortschreibung P52).</t>
         </is>
       </c>
       <c r="K103" s="41" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="J106" s="35" t="inlineStr">
         <is>
-          <t>Todesfälle × VSL + Verletzte × Behandlungskosten je Ereignisklasse.</t>
+          <t>Todesfälle als YLL × VOLY (MK 4.0; VSL nur Sensitivität — Fortschreibung P52) + Verletzte × Behandlungskosten je Ereignisklasse.</t>
         </is>
       </c>
       <c r="K106" s="35" t="inlineStr">
@@ -8328,8 +8328,6 @@
     </row>
     <row r="5" ht="15" customHeight="1" s="27"/>
     <row r="6" ht="15" customHeight="1" s="27"/>
-    <row r="7"/>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="27">
       <c r="A9" s="47" t="inlineStr">
         <is>
@@ -8350,7 +8348,7 @@
       </c>
       <c r="C10" s="50" t="inlineStr">
         <is>
-          <t>Mortalität (VSL je Todesfall) und Morbidität (Behandlungskosten je Fall) der Bevölkerung; partitioniert nach Ursachen: Hitze · Allergene · Infektion · UV · Vektoren · Luft · Extremereignisse — jeder Fall zählt genau einmal.</t>
+          <t>Mortalität (YLL × VOLY: verlorene Lebensjahre × Wert eines Lebensjahres, MK 4.0 — Fortschreibung P52) und Morbidität (Behandlungskosten je Fall) der Bevölkerung; partitioniert nach Ursachen: Hitze · Allergene · Infektion · UV · Vektoren · Luft · Extremereignisse — jeder Fall zählt genau einmal.</t>
         </is>
       </c>
     </row>
@@ -8362,7 +8360,7 @@
       </c>
       <c r="C11" s="50" t="inlineStr">
         <is>
-          <t>VSL (Nutzer-Setzung 3,5 Mio. €/Todesfall) · Behandlungskostensätze je Diagnose</t>
+          <t>YLL × VOLY (VOLY 160.800 €/Lebensjahr, Preisstand 2024, nach MK 4.0/Amann 2020a; VSL 3,5 / 4,7 / 6,19 Mio. €/Todesfall nur als Sensitivitäten — Fortschreibung P52) · Behandlungskostensätze je Diagnose</t>
         </is>
       </c>
     </row>
@@ -8402,8 +8400,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="27">
       <c r="A17" s="47" t="inlineStr">
         <is>
@@ -8476,8 +8472,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="27">
       <c r="A25" s="47" t="inlineStr">
         <is>
@@ -8550,8 +8544,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="27">
       <c r="A33" s="47" t="inlineStr">
         <is>
@@ -8624,8 +8616,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="27">
       <c r="A41" s="47" t="inlineStr">
         <is>
@@ -8698,8 +8688,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
-    <row r="48"/>
     <row r="49" ht="15" customHeight="1" s="27">
       <c r="A49" s="47" t="inlineStr">
         <is>
@@ -8772,8 +8760,6 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
     <row r="57" ht="15" customHeight="1" s="27">
       <c r="A57" s="47" t="inlineStr">
         <is>
@@ -8846,8 +8832,6 @@
         </is>
       </c>
     </row>
-    <row r="63"/>
-    <row r="64"/>
     <row r="65" ht="15" customHeight="1" s="27">
       <c r="A65" s="47" t="inlineStr">
         <is>
@@ -9203,7 +9187,7 @@
       </c>
       <c r="C16" s="53" t="inlineStr">
         <is>
-          <t>Volkswirtschaftlicher Schaden am Ort der Kommune (Wohlfahrtsperspektive, daher VSL 3,5 Mio. €). Alternative: fiskalische Sicht — nur Kosten des kommunalen Haushalts; dann entfallen VSL-Mortalität, private Sachschäden und BWS weitgehend.</t>
+          <t>Volkswirtschaftlicher Schaden am Ort der Kommune (Wohlfahrtsperspektive; Mortalität als YLL × VOLY nach MK 4.0 — Fortschreibung P52; VSL 3,5 Mio. € nur noch Sensitivität). Alternative: fiskalische Sicht — nur Kosten des kommunalen Haushalts; dann entfallen YLL-Mortalität, private Sachschäden und BWS weitgehend.</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F151"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="27" min="1" max="1"/>
@@ -13456,7 +13440,37 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="57" t="inlineStr">
+      <c r="A151" s="26" t="n">
+        <v>52</v>
+      </c>
+      <c r="B151" s="26" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="C151" s="26" t="inlineStr">
+        <is>
+          <t>Mortalitätsbewertung K1 (alle K1-Buchungsobjekte)</t>
+        </is>
+      </c>
+      <c r="D151" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E151" s="26" t="inlineStr">
+        <is>
+          <t>VSL 3,5 Mio. €/Fall → YLL × VOLY (MK 4.0, Amann 2020a: VOLY 160.800 €, Preisstand 2024); VSL 3,5/4,7/6,19 Mio. € als Sensitivitäten. Beschluss Review 2, umgesetzt Methodik-Bericht #95 Rev. 6 (Befund 50 der Gegenprüfung Rev. 5), 26.08.2026. Nachzug 26.08.2026 (zweiter Durchgang, Befund 70 der Runde-2-Gegenprüfung): Bewertungsbausteine der Zeilen ID 98 (Z103) und ID 101 (Z106) ebenfalls auf YLL × VOLY umgestellt; übrige K1-Zeilen ohne VSL-Nennung unverändert.</t>
+        </is>
+      </c>
+      <c r="F151" s="26" t="inlineStr">
+        <is>
+          <t>Fortschreibung Bewertungslogik (keine Kante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="57" t="inlineStr">
         <is>
           <t>147 Verbindungen ergänzt, 1 entfernt. Grundlage: Korrekturliste UBA-Abgleich (57 Punkte, entschieden Aug. 2026). Nur Verbindungen zwischen den 102 KWRA-Wirkungen (plus Fang-Sammelobjekt und Direktbuchungen in Konten); keine neuen Knoten, keine Sensitivitäten/Einflüsse/räumlichen Faktoren.</t>
         </is>

</xml_diff>